<commit_message>
Added July H2S data
</commit_message>
<xml_diff>
--- a/CO2xN/Porewater/Sulfide/2025/2025 July Porewater/Raw Data/20250714_LTREB_H2S_STD.xlsx
+++ b/CO2xN/Porewater/Sulfide/2025/2025 July Porewater/Raw Data/20250714_LTREB_H2S_STD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20346"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\microplate\Desktop\BioGeoChem_Microplates\LTREB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/blakleybd_si_edu/Documents/Documents/GitHub/GCREW/CO2xN/Porewater/Sulfide/2025/2025 July Porewater/Raw Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{951BF606-1041-4825-9791-8A7B532B5480}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{951BF606-1041-4825-9791-8A7B532B5480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8E34F4B-136F-4DC2-A935-43EAE0E2C170}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18885" windowHeight="11640" xr2:uid="{EC5EF5D1-F9F4-4E06-B5C3-1B303F8F9B16}"/>
+    <workbookView xWindow="2265" yWindow="1230" windowWidth="23955" windowHeight="13185" xr2:uid="{EC5EF5D1-F9F4-4E06-B5C3-1B303F8F9B16}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -494,6 +505,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -501,7 +513,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -872,6 +883,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -879,7 +891,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2030,16 +2041,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>423862</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>80962</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>185737</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>119062</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>61912</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>385762</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>71437</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2104,9 +2115,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2144,7 +2155,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2250,7 +2261,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2392,7 +2403,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>